<commit_message>
bars missing on notif fixed
</commit_message>
<xml_diff>
--- a/Functional_Test_Cases_trimmed.xlsx
+++ b/Functional_Test_Cases_trimmed.xlsx
@@ -15,12 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Setup" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Student'!$A$1:$I$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Registrar'!$A$1:$I$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Student'!$A$1:$I$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Registrar'!$A$1:$I$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Teacher'!$A$1:$I$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Program Head'!$A$1:$I$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Admin'!$A$1:$I$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Test Setup'!$A$1:$C$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Program Head'!$A$1:$I$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Admin'!$A$1:$I$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Test Setup'!$A$1:$C$50</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -581,7 +581,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Five steps: Submitted, Registrar, Teacher, Program Head, Scheduled. Finished steps show a gold ✓, the current step is navy, later steps are grey. Scheduled shows all five ticked.</t>
+          <t>Four steps: Submitted, Teacher, Program Head, Scheduled. There is no Registrar step. Finished steps show a gold ✓, the current step is navy, later steps are grey. Scheduled shows all four ticked.</t>
         </is>
       </c>
       <c r="G2" s="3" t="n"/>
@@ -618,7 +618,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Eight steps: Submitted, Registrar, Teacher, Program Head, Fee Assessment, Receipt, Checking, Scheduled. After the Program Head accepts, the current step is 'Fee Assessment'; after the Registrar assesses it, 'Receipt'; after upload, 'Checking'.</t>
+          <t>Seven steps: Submitted, Teacher, Program Head, Fee Assessment, Receipt, Checking, Scheduled. There is no Registrar step before the Teacher. After the Program Head accepts, the current step is 'Fee Assessment'; after the Registrar assesses it, 'Receipt'; after upload, 'Checking'.</t>
         </is>
       </c>
       <c r="G3" s="3" t="n"/>
@@ -908,12 +908,12 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Contact number changed.</t>
+          <t>Contact number changed. The request was rejected by the Program Head.</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>The request goes back to the reviewer who rejected it (Registrar, Teacher or Program Head) and shows the green message '✓ Request submitted successfully!' (the parent is not asked to verify again). The card shows the stage again and the reviewer sees a 'Resubmitted' label.</t>
+          <t>The request goes back to the Program Head (the only reviewer who rejects) and shows the green message '✓ Request submitted successfully!' (the parent is not asked to verify again). The card shows the stage again and the Program Head sees a 'Resubmitted' label.</t>
         </is>
       </c>
       <c r="G11" s="3" t="n"/>
@@ -950,7 +950,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>The page returns to the request. A green box '✓ Parent/guardian identity verified' appears with the document type and the scores. A yellow note says 'One step left. Your request has not been sent to the Registrar yet. Press Submit below to send it.' and a button 'Submit Request'. The card on My Requests still reads 'Not submitted yet'.</t>
+          <t>The page returns to the request. A green box '✓ Parent/guardian identity verified' appears with the document type and the scores. A yellow note says 'One step left. Your request has not been sent to the Subject Teacher yet. Press Submit below to send it.' and a button 'Submit Request'. The card on My Requests still reads 'Not submitted yet'.</t>
         </is>
       </c>
       <c r="G12" s="3" t="n"/>
@@ -986,7 +986,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>A red box 'Identity verification failed' lists what went wrong (or says 'The ID could not be confirmed, or the selfie did not match it.'), says the request will not reach the Registrar until it passes, and shows 'Try verification again'.</t>
+          <t>A red box 'Identity verification failed' lists what went wrong (or says 'The ID could not be confirmed, or the selfie did not match it.'), says the request will not reach the Subject Teacher until it passes, and shows 'Try verification again'.</t>
         </is>
       </c>
       <c r="G13" s="3" t="n"/>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>The button reads 'Submitting…'. The note changes to 'Your request is now with the Registrar.' The badge changes from 'Not submitted yet' to 'Submitted' and the request appears in the Registrar's queue. The Registrar receives an email 'New special exam request: &lt;student&gt; — &lt;code&gt;'.</t>
+          <t>The button reads 'Submitting…'. The note changes to 'Your request is now with the Subject Teacher.' The badge changes from 'Not submitted yet' to 'Submitted' and the request appears in the Teacher's queue (not the Registrar's). The Teacher receives an email 'New special exam request: &lt;student&gt; — &lt;code&gt;'. The Registrar receives nothing.</t>
         </is>
       </c>
       <c r="G15" s="3" t="n"/>
@@ -1086,17 +1086,17 @@
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Student A (see the 'Test Setup' sheet).
 2. Open the confirmation window.
 3. Click 'Yes, Withdraw'.
-4. Log in as the Registrar and look for it.</t>
+4. Log in as the Teacher and look for it.</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>A request waiting for the Registrar.</t>
+          <t>A request waiting for the Teacher.</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>The button reads 'Withdrawing…', then My Requests opens without that request. It is gone for good, including from the Registrar's queue. Pressing the browser's Back button shows 'This request is no longer available'.</t>
+          <t>The button reads 'Withdrawing…', then My Requests opens without that request. It is gone for good, including from the Teacher's queue. Pressing the browser's Back button shows 'This request is no longer available'.</t>
         </is>
       </c>
       <c r="G16" s="3" t="n"/>
@@ -1140,25 +1140,85 @@
       <c r="H17" s="3" t="n"/>
       <c r="I17" s="3" t="n"/>
     </row>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="56"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="104"/>
-    <row r="109"/>
-    <row r="112"/>
-    <row r="115"/>
-    <row r="118"/>
-    <row r="134"/>
-    <row r="140"/>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>TC-S-017</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Banner and Pop-ups</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Printed form reminder</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Student A (see the 'Test Setup' sheet).
+2. Look at the status banner at the top of the dashboard.</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>A student with an open submission window.</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>The banner says: 'Please also get the printed form from the Registrar's office and fill it in. The Registrar counts exam takers from it, and the Cashier marks it when you pay. Submitting here alone does not finish your request.'</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="n"/>
+      <c r="H18" s="3" t="n"/>
+      <c r="I18" s="3" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>TC-S-018</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Submit New Request</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Waived request skips the Registrar</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Student A (see the 'Test Setup' sheet).
+2. Submit an Excused request and pass the parent check.
+3. Log in as the Teacher and approve it.
+4. Log in as the Program Head and click 'Mark scheduled'.
+5. Log in as Student A and look at the card on My Requests.
+6. Log in as the Registrar and look at Payment Assessment.</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>An Excused request with a certificate.</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>The request goes Teacher, then Program Head, then Scheduled. The progress rail has four steps and never shows a Registrar step or 'Fee Assessment'. The request never appears for the Registrar and the Registrar receives no email.</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="n"/>
+      <c r="H19" s="3" t="n"/>
+      <c r="I19" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I17"/>
-  <conditionalFormatting sqref="H2:H17">
+  <autoFilter ref="A1:I19"/>
+  <conditionalFormatting sqref="H2:H19">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -1167,7 +1227,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Status" error="Choose Pass or Fail from the list." type="list">
+    <dataValidation sqref="H2:H19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1181,7 +1241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1250,29 +1310,29 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Pending Queue</t>
+          <t>Menu and home page</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Parent not verified: not listed</t>
+          <t>Registrar has no review queue</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Registrar A (see the 'Test Setup' sheet).
-2. Click the 'Pending Queue' tab.
-3. Look for Student 3's name.</t>
+2. Look at the left menu.
+3. Type the site address followed by /registrar and press Enter.</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Student 3 filled in the form but the parent check has not passed.</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Student 3 is NOT listed.</t>
+          <t>The menu has only 'Payment Assessment' and 'Parent List'. There is no 'Pending Queue' and no 'Verified History'. /registrar opens Payment Assessment.</t>
         </is>
       </c>
       <c r="G2" s="3" t="n"/>
@@ -1287,29 +1347,29 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Review Panel (right side)</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>'Parent check' - name matches the list</t>
+          <t>No alert or email when a student submits</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Registrar A (see the 'Test Setup' sheet).
-2. Click the 'Pending Queue' tab.
-3. Open the form of the student below.</t>
+2. Have Student 1 (paid) pass the parent check and press 'Submit Request'.
+3. Click the bell and open the Registrar's mailbox.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Student 1's parent list has 'Maria Luisa Dela Cruz' (Mother); the ID name read by Didit is 'MARIA LUISA DELA CRUZ'.</t>
+          <t>Student 1's form just submitted. It is now waiting for the Teacher.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>A green line 'Matches the mother on file', 'Name on the ID: …' and 'On the list: Mother Maria Luisa Dela Cruz'. A note says names can be written differently and you must compare them yourself.</t>
+          <t>The bell has no alert about this form and no email arrives. The Teacher is notified instead.</t>
         </is>
       </c>
       <c r="G3" s="3" t="n"/>
@@ -1324,29 +1384,29 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Review Panel (right side)</t>
+          <t>Payment Assessment</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>'Parent check' - name not on the list</t>
+          <t>Request before the Program Head accepts is not listed</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Registrar A (see the 'Test Setup' sheet).
-2. Click the 'Pending Queue' tab.
-3. Open the form of the student below.</t>
+2. Click the 'Payment Assessment' tab.
+3. Look for a student whose form is still with the Teacher or waiting for the Program Head's first approval.</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>List has Father 'Pedro Reyes'; ID name is 'Jose Santos'.</t>
+          <t>A paid request that the Program Head has not accepted yet.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>An orange line 'Not on the parent list' showing the ID name and the names on the list.</t>
+          <t>The student is NOT listed under 'Awaiting assessment' or 'Assessed'. The Registrar sees no ID photos, no certificate and no 'Parent check' anywhere.</t>
         </is>
       </c>
       <c r="G4" s="3" t="n"/>
@@ -1361,29 +1421,29 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Review Panel (right side)</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>'Parent check' - same name as the student</t>
+          <t>Fee assessment email (paid)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Registrar A (see the 'Test Setup' sheet).
-2. Click the 'Pending Queue' tab.
-3. Open the form of the student below.</t>
+2. Log in as the Program Head and accept Student 1's paid form.
+3. Open the Registrar's mailbox and the bell.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>The ID name is the student's own name (the student verified with their own ID).</t>
+          <t>Real mailbox for the Registrar.</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>A red line 'Same name as the student. They may have verified as their own parent.' It is only a warning: the Verify button still works.</t>
+          <t>An email 'Fee assessment needed: &lt;student&gt; — &lt;code&gt;' with a button 'Assess fees' and the progress bar 'Step 4 of 7 · Fee Assessment'. The bell shows the student awaiting payment assessment.</t>
         </is>
       </c>
       <c r="G5" s="3" t="n"/>
@@ -1398,29 +1458,29 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Review Panel (right side)</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Registrar does not see ID photos or the certificate</t>
+          <t>Waived (excused) request never reaches the Registrar</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Registrar A (see the 'Test Setup' sheet).
-2. Click the 'Pending Queue' tab.
-3. Click an excused student with an uploaded certificate.</t>
+2. Log in as the Program Head and click 'Mark scheduled' on Student 8's excused form.
+3. Open the Registrar's mailbox, the bell and Payment Assessment.</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Student 8 uploaded a medical certificate.</t>
+          <t>Student 8's Excused request.</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>There is NO 'Documents' section and no ID photo or selfie. Only the form details, the parent check result and History.</t>
+          <t>The Registrar gets no email and no alert, and Student 8 is not listed in Payment Assessment.</t>
         </is>
       </c>
       <c r="G6" s="3" t="n"/>
@@ -1435,30 +1495,29 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Verify (single form)</t>
+          <t>Payment Assessment</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>'Verify &amp; Forward to Teacher'</t>
+          <t>'Mark assessed' for a student</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Registrar A (see the 'Test Setup' sheet).
-2. Click the 'Pending Queue' tab.
-3. Click Student 1's name.
-4. Click the gold 'Verify &amp; Forward to Teacher' button.</t>
+2. Click the 'Payment Assessment' tab.
+3. Click 'Mark assessed' on Student 10's row.</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Student 1's only form.</t>
+          <t>Student 10 with 2 subjects, fee ₱200 each.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>The button reads 'Processing…', then the form and Student 1's row disappear and the right side goes back to 'Select a student…'. No error.</t>
+          <t>The button reads 'Recording…'. The row leaves 'Awaiting assessment' and appears under 'Assessed' with amount ₱400 and the date ('Just now' right after). The tab numbers update.</t>
         </is>
       </c>
       <c r="G7" s="3" t="n"/>
@@ -1473,29 +1532,29 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Verify (single form)</t>
+          <t>Payment Assessment</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Emails after verifying</t>
+          <t>Student is told the amount (email)</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Registrar A (see the 'Test Setup' sheet).
-2. Verify Student 1's form.
-3. Open the mailboxes of Student 1 and the Teacher.</t>
+2. Mark Student 10 as assessed.
+3. Open Student 10's mailbox.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Real mailboxes for Student 1 and the Teacher.</t>
+          <t>Real mailbox for Student 10.</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Student 1 receives 'Update: the Registrar verified your request for &lt;subject code&gt;' (waiting for the teacher). The Teacher receives 'Waiting for your approval: &lt;student&gt; — &lt;subject code&gt;' with a 'Review request' button.</t>
+          <t>One email 'Your special exam fees are assessed' with 'Amount to pay: ₱400 for 2 subjects' and a button 'Upload receipt'.</t>
         </is>
       </c>
       <c r="G8" s="3" t="n"/>
@@ -1510,244 +1569,15 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Verify all</t>
+          <t>Parent List</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>'Verify all N forms'</t>
+          <t>'Replace the list'</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Registrar A (see the 'Test Setup' sheet).
-2. Click the 'Pending Queue' tab.
-3. Click Student 2's name.
-4. Click 'Verify all 2 forms'.</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Student 2 has 2 forms.</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>The button reads 'Verifying…' and is disabled. Both forms and Student 2's row disappear. Verified History shows both as 'Verified by Registrar' and the teachers are notified.</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>TC-R-009</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Reject</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>'Confirm reject' without a reason</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Registrar A (see the 'Test Setup' sheet).
-2. Click the 'Pending Queue' tab.
-3. Click Student 1's name.
-4. Click 'Reject'.
-5. Try to click 'Confirm reject' without choosing a reason.</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>No reason chosen.</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>'Confirm reject' cannot be clicked. Nothing is rejected.</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>TC-R-010</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Reject</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Reject with a ready-made reason</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Registrar A (see the 'Test Setup' sheet).
-2. Click the 'Pending Queue' tab.
-3. Click a student's name.
-4. Click 'Reject'.
-5. Click one reason.
-6. Click 'Confirm reject'.
-7. Repeat for two more forms with different reasons.</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Reasons, one per form: 'Wrong or incomplete student details'; 'Student number does not match school records'; 'Wrong subject or section selected'.</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>The chosen reason turns red. After 'Confirm reject' (it reads 'Rejecting…') the form disappears from the queue.</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>TC-R-011</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Reject</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Student is emailed about the rejection</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Registrar A (see the 'Test Setup' sheet).
-2. Reject Student 1's form.
-3. Open Student 1's mailbox.</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>Real mailbox for Student 1.</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Student 1 receives 'Your special exam request for &lt;subject code&gt; was rejected' with the Reason, and a note that they can fix it and resubmit.</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n"/>
-      <c r="I12" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>TC-R-012</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Payment Assessment</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>'Mark assessed' for a student</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Registrar A (see the 'Test Setup' sheet).
-2. Click the 'Payment Assessment' tab.
-3. Click 'Mark assessed' on Student 10's row.</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Student 10 with 2 subjects, fee ₱200 each.</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>The button reads 'Recording…'. The row leaves 'Awaiting assessment' and appears under 'Assessed' with amount ₱400 and the date ('Just now' right after). The tab numbers update.</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n"/>
-      <c r="I13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>TC-R-013</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Payment Assessment</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Student is told the amount (email)</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Registrar A (see the 'Test Setup' sheet).
-2. Mark Student 10 as assessed.
-3. Open Student 10's mailbox.</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>Real mailbox for Student 10.</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>One email 'Your special exam fees are assessed' with 'Amount to pay: ₱400 for 2 subjects' and a button 'Upload receipt'.</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>TC-R-014</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Parent List</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>'Replace the list'</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Registrar A (see the 'Test Setup' sheet).
 2. Click the 'Parent List' tab.
@@ -1755,37 +1585,23 @@
 4. Click 'Replace the list'.</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>A correct workbook (3 students, 5 parents).</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>The button reads 'Saving…', then a green message 'Saved: 3 students, 5 parents and guardians.' The table on the left shows the new list, and the file box is cleared.</t>
         </is>
       </c>
-      <c r="G15" s="3" t="n"/>
-      <c r="H15" s="3" t="n"/>
-      <c r="I15" s="3" t="n"/>
-    </row>
-    <row r="34"/>
-    <row r="51"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="57"/>
-    <row r="59"/>
-    <row r="61"/>
-    <row r="69"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="83"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="130"/>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I15"/>
-  <conditionalFormatting sqref="H2:H15">
+  <autoFilter ref="A1:I9"/>
+  <conditionalFormatting sqref="H2:H9">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -1794,7 +1610,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Status" error="Choose Pass or Fail from the list." type="list">
+    <dataValidation sqref="H2:H9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1894,7 +1710,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Student 4 has a form (Verified by Registrar) for a subject that belongs to Teacher B, not Teacher A.</t>
+          <t>Student 4 has a submitted form (parent verified) for a subject that belongs to Teacher B, not Teacher A.</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -1914,52 +1730,89 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
+          <t>Pending Queue</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Form not submitted yet is not listed</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Teacher A (see the 'Test Setup' sheet).
+2. Click the 'Pending Queue' tab.
+3. Look for Student 3's name.</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Student 3 filled in the form for Teacher A's subject, but the parent check has not passed (or the student has not pressed Submit).</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Student 3 is NOT listed, and the 'Pending Queue' badge and the bell do not count the form.</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>TC-T-003</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
           <t>Review Panel (right side)</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Teacher does not see documents or the parent check</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Teacher A (see the 'Test Setup' sheet).
 2. Click the 'Pending Queue' tab.
 3. Click a student whose form has uploaded files (an Excused request with a certificate).</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Student 7 uploaded a medical certificate.</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>There is NO 'Documents' section and NO 'Parent check' section (no ID photos, no certificate). Only form details and History.</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>TC-T-003</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TC-T-004</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Approve (single form)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>'Approve &amp; Forward to Program Head' - Paid form</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Teacher A (see the 'Test Setup' sheet).
 2. Click the 'Pending Queue' tab.
@@ -1967,37 +1820,37 @@
 4. Click the gold 'Approve &amp; Forward to Program Head' button.</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Student 1's Paid form (the student's only pending form).</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>The button briefly reads 'Processing…'. Then the form disappears, Student 1's row disappears from the list, the right side returns to 'Select a student…', and no error is shown.</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>TC-T-004</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TC-T-005</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Approve (single form)</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Approved form appears in Reviewed History</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Teacher A (see the 'Test Setup' sheet).
 2. Approve Student 1's form (see the previous test cases).
@@ -2005,37 +1858,37 @@
 4. Look at the top of the table.</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>A row for Student 1 with status 'Approved by Teacher' is at the top of the table.</t>
         </is>
       </c>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>TC-T-005</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>TC-T-006</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Approve (single form)</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Program Head receives the approved form</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Teacher A (see the 'Test Setup' sheet).
 2. Approve Student 1's form.
@@ -2043,90 +1896,51 @@
 4. Open the Program Head's first-approval queue and the bell.</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Program Head of the subject's department.</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Student 1's request is in the Program Head's queue, and the bell says the request is awaiting first approval.</t>
         </is>
       </c>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>TC-T-006</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TC-T-007</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Approve (single form)</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Emails after approval</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Teacher A (see the 'Test Setup' sheet).
 2. Approve Student 1's form.
 3. Open the student's mailbox and the Program Head's mailbox.</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Real mailboxes for Student 1 and the Program Head.</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Student 1 receives an email titled 'Update: your teacher approved your request for &lt;subject code&gt;' (it says the request is now with the Program Head). The Program Head also receives a notification email.</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>TC-T-007</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Reject</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>'Confirm reject' without a reason</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Teacher A (see the 'Test Setup' sheet).
-2. Click the 'Pending Queue' tab.
-3. Click Student 1's name.
-4. Click 'Reject'.
-5. Try to click 'Confirm reject' without choosing a reason.</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>No reason chosen.</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>'Confirm reject' cannot be clicked (greyed out). Nothing is rejected.</t>
         </is>
       </c>
       <c r="G8" s="3" t="n"/>
@@ -2141,93 +1955,15 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Reject</t>
+          <t>Approve all</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Reject with a ready-made reason</t>
+          <t>'Approve all N forms'</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Teacher A (see the 'Test Setup' sheet).
-2. Click the 'Pending Queue' tab.
-3. Click a student's name.
-4. Click 'Reject'.
-5. Click one reason.
-6. Click 'Confirm reject'.
-7. Repeat for three more forms, using a different reason each time.</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Reasons to use, one per form: 'Not enrolled in this subject'; 'Absence not valid for a special exam'; 'Insufficient justification'; 'Already took the exam'.</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>The chosen reason turns red. After 'Confirm reject' (it reads 'Rejecting…' briefly) the form disappears from the queue.</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>TC-T-009</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Reject</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Student is told about the rejection (email)</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Teacher A (see the 'Test Setup' sheet).
-2. Reject Student 1's form with the reason 'Insufficient justification'.
-3. Open Student 1's mailbox.</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Real mailbox for Student 1.</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Student 1 receives an email titled 'Your special exam request for &lt;subject code&gt; was rejected' that shows the Reason.</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>TC-T-010</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Approve all</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>'Approve all N forms'</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Teacher A (see the 'Test Setup' sheet).
 2. Click the 'Pending Queue' tab.
@@ -2235,29 +1971,95 @@
 4. Click 'Approve all 2 forms'.</t>
         </is>
       </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Student 2 has 2 pending forms.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>The button reads 'Approving…' and is disabled. Then both forms and Student 2's row disappear. Reviewed History shows both as 'Approved by Teacher'. The student gets notified.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TC-T-009</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Review Panel (right side)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Teacher has no Reject button</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Teacher A (see the 'Test Setup' sheet).
+2. Click the 'Pending Queue' tab.
+3. Click a student's name.
+4. Look at the buttons on each form, then click 'Approve all' if it is shown.</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>A student with a pending form.</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Each form has only the gold 'Approve &amp; Forward to Program Head' button. There is NO 'Reject' button and no rejection reason box.</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="n"/>
+      <c r="H10" s="3" t="n"/>
+      <c r="I10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>TC-T-010</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Teacher is told about a new submission</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Teacher A (see the 'Test Setup' sheet).
+2. Have a student press 'Submit Request' for Teacher A's subject.
+3. Click the bell and open Teacher A's mailbox.</t>
+        </is>
+      </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Student 2 has 2 pending forms.</t>
+          <t>Real mailbox for Teacher A.</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>The button reads 'Approving…' and is disabled. Then both forms and Student 2's row disappear. Reviewed History shows both as 'Approved by Teacher'. The student gets notified.</t>
+          <t>The bell says '&lt;student&gt; submitted a request for &lt;code&gt; — it is ready for your approval.' An email 'New special exam request: &lt;student&gt; — &lt;code&gt;' with the heading 'New request to approve' and a button 'Review request' arrives.</t>
         </is>
       </c>
       <c r="G11" s="3" t="n"/>
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="3" t="n"/>
     </row>
-    <row r="25"/>
-    <row r="27"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="48"/>
-    <row r="54"/>
   </sheetData>
   <autoFilter ref="A1:I11"/>
   <conditionalFormatting sqref="H2:H11">
@@ -2269,7 +2071,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Status" error="Choose Pass or Fail from the list." type="list">
+    <dataValidation sqref="H2:H11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2283,7 +2085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2427,15 +2229,163 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
+          <t>First Approval (panel)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>'Parent check' - name matches the list</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Program Head A (see the 'Test Setup' sheet).
+2. Click the 'First Approval' tab.
+3. Open the form of the student below.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Student 1's parent list has 'Maria Luisa Dela Cruz' (Mother); the ID name read by Didit is 'MARIA LUISA DELA CRUZ'.</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>A green line 'Matches the mother on file', 'Name on the ID: …' and 'On the list: Mother Maria Luisa Dela Cruz'. A note says names can be written differently and you must compare them yourself.</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TC-P-004</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>First Approval (panel)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>'Parent check' - name not on the list</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Program Head A (see the 'Test Setup' sheet).
+2. Click the 'First Approval' tab.
+3. Open the form of the student below.</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>List has Father 'Pedro Reyes'; ID name is 'Jose Santos'.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>An orange line 'Not on the parent list' showing the ID name and the names on the list. Only the Program Head sees this; the Teacher and the Registrar do not.</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TC-P-005</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>First Approval (panel)</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>'Parent check' - same name as the student</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Program Head A (see the 'Test Setup' sheet).
+2. Click the 'First Approval' tab.
+3. Open the form of the student below.</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>The ID name is the student's own name (the student verified with their own ID).</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>A red line 'Same name as the student. They may have verified as their own parent.' It is only a warning: 'Accept' still works.</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>TC-P-006</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>First Approval (panel)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Only the Teacher's approval is shown</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Program Head A (see the 'Test Setup' sheet).
+2. Click the 'First Approval' tab.
+3. Look at the line under the exam type on a form.</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>A form approved by the Teacher.</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>A green tick 'Teacher approved'. There is no 'Registrar verified' tick.</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TC-P-007</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
           <t>Accept (first approval)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>'Accept' a paid form</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Program Head A (see the 'Test Setup' sheet).
 2. Click the 'First Approval' tab.
@@ -2443,37 +2393,37 @@
 4. Click 'Accept'.</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Student 1's only form (Paid).</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>The button reads 'Processing…', then the form and the student's row disappear. No error.</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>TC-P-004</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="G8" s="3" t="n"/>
+      <c r="H8" s="3" t="n"/>
+      <c r="I8" s="3" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TC-P-008</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Accept (first approval)</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Student is told the form was accepted (paid)</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Program Head A (see the 'Test Setup' sheet).
 2. Accept Student 1's form.
@@ -2481,37 +2431,37 @@
 4. Log in as Student 1 and open My Requests.</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Real mailbox for Student 1.</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Student 1 gets 'Your special exam request for &lt;code&gt; was accepted' (go to the Registrar for fee assessment, pay at the Cashier, then upload the receipt). The request card reads 'Awaiting Fee Assessment'.</t>
         </is>
       </c>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>TC-P-005</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TC-P-009</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Accept (first approval)</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>'Mark scheduled' an excused form</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Program Head A (see the 'Test Setup' sheet).
 2. Click the 'First Approval' tab.
@@ -2519,37 +2469,37 @@
 4. Click 'Mark scheduled'.</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Student 7's Excused form.</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>The form disappears. It is now Scheduled (no receipt step) and appears on 'Accepted Students'. Student 7 gets 'Your special exam for &lt;code&gt; is scheduled'.</t>
         </is>
       </c>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>TC-P-006</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="G10" s="3" t="n"/>
+      <c r="H10" s="3" t="n"/>
+      <c r="I10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>TC-P-010</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Accept all</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>'Accept all N forms'</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Program Head A (see the 'Test Setup' sheet).
 2. Click the 'First Approval' tab.
@@ -2557,37 +2507,37 @@
 4. Click 'Accept all 2 forms'.</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Student 2 has 1 paid and 1 excused form.</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>The button reads 'Accepting…'. Both forms and the row disappear. The paid form goes to fee assessment; the excused form becomes Scheduled. The student gets the matching emails.</t>
         </is>
       </c>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>TC-P-007</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
+      <c r="I11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TC-P-011</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Reject (first approval)</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Reject with a ready-made reason</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Program Head A (see the 'Test Setup' sheet).
 2. Click the 'First Approval' tab.
@@ -2596,37 +2546,37 @@
 5. Click 'Confirm reject'.</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Reason: Details do not match records.</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>The chosen reason turns red. After 'Confirm reject' (it reads 'Rejecting…') the form disappears.</t>
         </is>
       </c>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
-      <c r="I8" s="3" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>TC-P-008</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
+      <c r="I12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TC-P-012</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Return for re-verification</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Return with a ready-made reason</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Program Head A (see the 'Test Setup' sheet).
 2. Click the 'First Approval' tab.
@@ -2636,37 +2586,37 @@
 6. Click 'Return to student'.</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>Reason: Face does not match the ID.</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>The button reads 'Returning…'. The form disappears from First Approval and the badge/bell numbers go down. The request is NOT rejected.</t>
         </is>
       </c>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>TC-P-009</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TC-P-013</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Return for re-verification</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>What the student sees after a return</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Program Head A (see the 'Test Setup' sheet).
 2. Return a form.
@@ -2674,37 +2624,37 @@
 4. Log in as that student and open My Requests and the bell.</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>Real mailbox for the student.</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>Email 'Action needed: your parent or guardian must verify again (&lt;code&gt;)' with the reason. The request card reads 'Verify parent again' with a strip 'Your Program Head asked your parent or guardian to verify again' and a 'See why' button. The bell says 'Action needed: your Program Head asked your parent or guardian to verify again for &lt;code&gt;.'</t>
         </is>
       </c>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>TC-P-010</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="G14" s="3" t="n"/>
+      <c r="H14" s="3" t="n"/>
+      <c r="I14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>TC-P-014</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Second Approval (receipts)</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>'Confirm receipt and schedule'</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Program Head A (see the 'Test Setup' sheet).
 2. Click the 'Second Approval' tab.
@@ -2712,37 +2662,37 @@
 4. Click 'Confirm receipt and schedule'.</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>Student 9's paid form with a receipt.</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>The button reads 'Confirming…'. The form disappears and the request becomes Scheduled. It now appears on 'Accepted Students'.</t>
         </is>
       </c>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>TC-P-011</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TC-P-015</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Second Approval (receipts)</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Student is told the exam is scheduled</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Program Head A (see the 'Test Setup' sheet).
 2. Confirm Student 9's receipt.
@@ -2750,37 +2700,37 @@
 4. Log in as Student 9.</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>Real mailbox for Student 9.</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Email 'Your special exam for &lt;code&gt; is scheduled' with the exam date, venue and what to bring (or a note to open EXAMFLOW if not set). The request card shows 'Scheduled' and the bell says 'Your special exam for &lt;code&gt; is scheduled.'</t>
         </is>
       </c>
-      <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n"/>
-      <c r="I12" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>TC-P-012</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="G16" s="3" t="n"/>
+      <c r="H16" s="3" t="n"/>
+      <c r="I16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>TC-P-016</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Second Approval (receipts)</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Reject a receipt</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Program Head A (see the 'Test Setup' sheet).
 2. Click the 'Second Approval' tab.
@@ -2790,37 +2740,37 @@
 6. Click 'Confirm reject'.</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>Reason: Blurred or unreadable receipt.</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>The form disappears from this page. The request goes back to 'accepted' so the student can upload again.</t>
         </is>
       </c>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n"/>
-      <c r="I13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>TC-P-013</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="3" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>TC-P-017</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Accepted Students</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Export to Excel</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Program Head A (see the 'Test Setup' sheet).
 2. Click the 'Accepted Students' tab.
@@ -2828,37 +2778,37 @@
 4. Open the downloaded file.</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Scheduled students: some paid, some excused, in different subjects.</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>A file 'Special-Exam-Application_&lt;today's date&gt;.xlsx' downloads with three sheets: 'PAID SPECIAL EXAM', 'WAIVED FEE (VALID REASON)' and 'Summary'. The paid and waived sheets have the columns Date of Application, Student Name, Section, Course/Subject Title, Course/Subject Code, Program/Strand (the waived sheet also has 'Reason'). The Summary lists each subject code with its count and a TOTAL.</t>
         </is>
       </c>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>TC-P-014</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="G18" s="3" t="n"/>
+      <c r="H18" s="3" t="n"/>
+      <c r="I18" s="3" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>TC-P-018</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Exam Periods</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Save a term with a submission window</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Program Head A (see the 'Test Setup' sheet).
 2. Click the 'Exam Periods' tab.
@@ -2869,37 +2819,37 @@
 7. Click 'Yes, set it'.</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>Semester 1st; Term Prelim; start date today; 7 days.</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>A note shows 'Submissions close on &lt;date&gt; (7 days).' The confirmation window shows 'New: Opens &lt;date&gt; · 7 days (closes &lt;date&gt;)'. After confirming: green 'Window saved and set active.' and the summary card shows the term as Active.</t>
         </is>
       </c>
-      <c r="G15" s="3" t="n"/>
-      <c r="H15" s="3" t="n"/>
-      <c r="I15" s="3" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>TC-P-015</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="G19" s="3" t="n"/>
+      <c r="H19" s="3" t="n"/>
+      <c r="I19" s="3" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>TC-P-019</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>Exam Periods</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>Save the exam schedule</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Program Head A (see the 'Test Setup' sheet).
 2. Click the 'Exam Periods' tab.
@@ -2908,38 +2858,23 @@
 5. Click 'Yes, set it'.</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>Exam date: 14 days from today; Location: Room 401; What to bring: Valid ID, blue pen.</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>A green message 'Schedule saved. Students can now see it.' and the summary card shows the date. Students see the schedule on their dashboard and bell.</t>
         </is>
       </c>
-      <c r="G16" s="3" t="n"/>
-      <c r="H16" s="3" t="n"/>
-      <c r="I16" s="3" t="n"/>
-    </row>
-    <row r="33"/>
-    <row r="49"/>
-    <row r="57"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="68"/>
-    <row r="75"/>
-    <row r="85"/>
-    <row r="88"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="99"/>
-    <row r="121"/>
-    <row r="133"/>
-    <row r="140"/>
+      <c r="G20" s="3" t="n"/>
+      <c r="H20" s="3" t="n"/>
+      <c r="I20" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I16"/>
-  <conditionalFormatting sqref="H2:H16">
+  <autoFilter ref="A1:I20"/>
+  <conditionalFormatting sqref="H2:H20">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -2948,7 +2883,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Status" error="Choose Pass or Fail from the list." type="list">
+    <dataValidation sqref="H2:H20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2962,7 +2897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3036,15 +2971,15 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Admin approves as Registrar</t>
+          <t>Admin approves as Teacher</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
           <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Admin A (see the 'Test Setup' sheet).
 2. Click the 'Requests' tab in the top menu.
-3. Click 'Waiting for Registrar' and 'Open as Registrar'.
-4. Verify the request as the Registrar would.
+3. Click 'Waiting for Teacher' and 'Open as Teacher'.
+4. Approve the request as the Teacher would.
 5. Open the request's History.</t>
         </is>
       </c>
@@ -3055,7 +2990,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>The request moves on to the Teacher stage. Its History shows the step marked '(by Admin)'. The request now appears under 'Waiting for Teacher' on the Requests page.</t>
+          <t>The request moves on to the Program Head stage. Its History shows the step marked '(by Admin)'. The request now appears under 'Waiting for Program Head' on the Requests page.</t>
         </is>
       </c>
       <c r="G2" s="3" t="n"/>
@@ -3179,7 +3114,7 @@
       </c>
       <c r="G5" s="3" t="n"/>
       <c r="H5" s="3" t="n"/>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>NEEDS CHECKING: The error appears in a red box at the top of the Users page, which sits BEHIND the dark overlay of the Create window, so it may be hard to see. The window also stays open.</t>
         </is>
@@ -3643,25 +3578,46 @@
       <c r="H17" s="3" t="n"/>
       <c r="I17" s="3" t="n"/>
     </row>
-    <row r="40"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="88"/>
-    <row r="96"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="106"/>
-    <row r="121"/>
-    <row r="142"/>
-    <row r="145"/>
-    <row r="149"/>
-    <row r="156"/>
-    <row r="179"/>
-    <row r="186"/>
-    <row r="194"/>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>TC-A-017</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Requests</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Stage list has no Registrar review</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>1. Open the EXAMFLOW website (www.examflow.me) and log in as Admin A (see the 'Test Setup' sheet).
+2. Click the 'Requests' tab in the top menu.
+3. Look at the stage names above the list.</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Requests at several stages.</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>The stages are 'Waiting for Teacher', 'Waiting for Program Head', 'Waiting for assessment', 'Waiting for payment', 'Receipt to verify' and 'Rejected'. There is no 'Waiting for Registrar'. A paid request waiting for assessment opens 'Payment assessment'.</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="n"/>
+      <c r="H18" s="3" t="n"/>
+      <c r="I18" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I17"/>
-  <conditionalFormatting sqref="H2:H17">
+  <autoFilter ref="A1:I18"/>
+  <conditionalFormatting sqref="H2:H18">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3670,7 +3626,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Status" error="Choose Pass or Fail from the list." type="list">
+    <dataValidation sqref="H2:H18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3684,7 +3640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3807,7 +3763,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Requests for Student A at: just filled in; submitted; verified by the Registrar; approved by the Teacher; accepted (paid, not assessed); accepted (paid, assessed); receipt uploaded; scheduled; rejected; returned by the Program Head; and one from an earlier term.</t>
+          <t>Requests for Student A at: just filled in; submitted (waiting for the Teacher); approved by the Teacher; accepted (paid, not assessed); accepted (paid, assessed); receipt uploaded; scheduled; rejected by the Program Head; returned by the Program Head; and one from an earlier term.</t>
         </is>
       </c>
     </row>
@@ -3909,7 +3865,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Paid request, parent passed the check and the student pressed Submit (1 form waiting for the Registrar). Leave Contact number empty. Parent list: Mother 'Maria Luisa Dela Cruz'.</t>
+          <t>Paid request accepted by the Program Head, not yet assessed (also used to check there is no Registrar queue). Leave Contact number empty.</t>
         </is>
       </c>
     </row>
@@ -3921,12 +3877,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Student 2</t>
+          <t>Student 8</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Two requests, both submitted and waiting for the Registrar.</t>
+          <t>An Excused request with a medical certificate, accepted/scheduled by the Program Head (it must never appear for the Registrar).</t>
         </is>
       </c>
     </row>
@@ -3938,12 +3894,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Student 3</t>
+          <t>Student 10</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Request filled in but the parent check has not passed.</t>
+          <t>Two paid requests accepted by the Program Head (not assessed), student number 2024-00010, BSIT 3rd year, section BSIT 3-301.</t>
         </is>
       </c>
     </row>
@@ -3955,12 +3911,12 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Student 8</t>
+          <t>Parent list file</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>An Excused request with a medical certificate, waiting for the Registrar; also accepted/scheduled by the Program Head for the 'excused never appears' case.</t>
+          <t>A correct .xlsx file with the columns Student Number, Student Name, Father, Mother, Guardian, Guardian Relationship, plus broken files (no header row, repeated student number, a student with no parent, a .pdf, a text file renamed .xlsx, a file over 10 MB).</t>
         </is>
       </c>
     </row>
@@ -3972,12 +3928,12 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Student 10</t>
+          <t>Mailboxes</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Two paid requests accepted by the Program Head (not assessed), student number 2024-00010, BSIT 3rd year, section BSIT 3-301.</t>
+          <t>Real inboxes for the students and the Teacher, to check the emails.</t>
         </is>
       </c>
     </row>
@@ -3989,46 +3945,46 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Parent list file</t>
+          <t>Note</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>A correct .xlsx file with the columns Student Number, Student Name, Father, Mother, Guardian, Guardian Relationship, plus broken files (no header row, repeated student number, a student with no parent, a .pdf, a text file renamed .xlsx, a file over 10 MB).</t>
+          <t>Many tests change data (assess, replace the parent list). Use a test system and create fresh requests before repeating a test. Test cases name people as examples; use any account that matches the description.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Registrar</t>
+          <t>Teacher</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Mailboxes</t>
+          <t>Teacher A</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Real inboxes for the students and the Teacher, to check the emails.</t>
+          <t>An active Subject Teacher account assigned to at least two subjects (Subject A1, Subject A2) and to a department.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Registrar</t>
+          <t>Teacher</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Note</t>
+          <t>Teacher B</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Many tests change data (verify, reject, assess, replace the parent list). Use a test system and create fresh requests before repeating a test. Test cases name people as examples; use any account that matches the description.</t>
+          <t>A second Subject Teacher account with its own subject (used to check that Teacher A cannot see Teacher B's students).</t>
         </is>
       </c>
     </row>
@@ -4040,12 +3996,12 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Teacher A</t>
+          <t>Student 3</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>An active Subject Teacher account assigned to at least two subjects (Subject A1, Subject A2) and to a department.</t>
+          <t>Request for Teacher A's subject that is filled in, but the parent check has not passed (or the student has not pressed Submit).</t>
         </is>
       </c>
     </row>
@@ -4057,12 +4013,12 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Teacher B</t>
+          <t>Program Head</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>A second Subject Teacher account with its own subject (used to check that Teacher A cannot see Teacher B's students).</t>
+          <t>An active Program Head account for the same department (to check forwarded requests, and to activate a new term).</t>
         </is>
       </c>
     </row>
@@ -4074,12 +4030,12 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Registrar</t>
+          <t>Active exam term</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>An active Registrar account (to verify requests so they reach the teacher).</t>
+          <t>The Program Head must have an active term. Requests only show in the teacher pages for the active term.</t>
         </is>
       </c>
     </row>
@@ -4091,12 +4047,12 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Program Head</t>
+          <t>Student 1</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>An active Program Head account for the same department (to check forwarded requests, and to activate a new term).</t>
+          <t>Paid request for Subject A1, submitted (parent verified and the student pressed Submit), waiting for the Teacher. 1 form. Leave the Contact number empty.</t>
         </is>
       </c>
     </row>
@@ -4108,12 +4064,12 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Active exam term</t>
+          <t>Student 2</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>The Program Head must have an active term. Requests only show in the teacher pages for the active term.</t>
+          <t>Two requests (Subject A1 paid and Subject A2 paid or excused), both submitted and waiting for the Teacher.</t>
         </is>
       </c>
     </row>
@@ -4125,12 +4081,12 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Student 1</t>
+          <t>Student 4</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Paid request for Subject A1, status 'Verified by Registrar' (1 form). Leave the Contact number empty.</t>
+          <t>Submitted request (parent verified) for Teacher B's subject.</t>
         </is>
       </c>
     </row>
@@ -4142,12 +4098,12 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Student 2</t>
+          <t>Student 7</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Two requests (Subject A1 paid and Subject A2 paid or excused), both 'Verified by Registrar'.</t>
+          <t>Excused request with a reason and an uploaded certificate, submitted and waiting for the Teacher, for Teacher A's subject.</t>
         </is>
       </c>
     </row>
@@ -4159,12 +4115,12 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Student 4</t>
+          <t>Mailboxes</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Request 'Verified by Registrar' for Teacher B's subject.</t>
+          <t>Real email inboxes for the students and the Program Head, to check the emails.</t>
         </is>
       </c>
     </row>
@@ -4176,46 +4132,46 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Student 7</t>
+          <t>Note</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Excused request with a reason and an uploaded certificate, 'Verified by Registrar', for Teacher A's subject.</t>
+          <t>Many tests change data (approve). Create fresh requests, or reset them, before repeating a test. Test cases refer to these students by name; use any students that match the description.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Teacher</t>
+          <t>Program Head</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Mailboxes</t>
+          <t>Program Head A</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Real email inboxes for the students and the Program Head, to check the emails.</t>
+          <t>An active Program Head account assigned to Department X.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Teacher</t>
+          <t>Program Head</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Note</t>
+          <t>Other roles</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Many tests change data (approve/reject). Create fresh requests, or reset them, before repeating a test. Test cases refer to these students by name; use any students that match the description.</t>
+          <t>Active accounts for Student, Subject Teacher, Registrar and Admin. A second Program Head or the Admin to try the 'two windows' cases.</t>
         </is>
       </c>
     </row>
@@ -4227,12 +4183,12 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Program Head A</t>
+          <t>Department Y</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>An active Program Head account assigned to Department X.</t>
+          <t>A second department with its own subjects and requests (to check that Program Head A cannot see them).</t>
         </is>
       </c>
     </row>
@@ -4244,12 +4200,12 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Other roles</t>
+          <t>Active exam term</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Active accounts for Student, Subject Teacher, Registrar and Admin. A second Program Head or the Admin to try the 'two windows' cases.</t>
+          <t>An active term with a submission window and a saved exam schedule.</t>
         </is>
       </c>
     </row>
@@ -4261,12 +4217,12 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Department Y</t>
+          <t>Didit</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>A second department with its own subjects and requests (to check that Program Head A cannot see them).</t>
+          <t>Verified parent checks need Didit. In a test system use Didit's test mode; ask the developer how photos behave there.</t>
         </is>
       </c>
     </row>
@@ -4278,12 +4234,12 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Active exam term</t>
+          <t>Student 1</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>An active term with a submission window and a saved exam schedule.</t>
+          <t>Paid request in Department X, approved by the Teacher, parent verified (1 form).</t>
         </is>
       </c>
     </row>
@@ -4295,12 +4251,12 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Didit</t>
+          <t>Parent list</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Verified parent checks need Didit. In a test system use Didit's test mode; ask the developer how photos behave there.</t>
+          <t>A parent list uploaded by the Registrar: Student 1's Mother is 'Maria Luisa Dela Cruz'; another student's Father is 'Pedro Reyes' (with Didit reading a different name, 'Jose Santos'); and one student whose ID name is the student's own name.</t>
         </is>
       </c>
     </row>
@@ -4312,12 +4268,12 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Student 1</t>
+          <t>Student 2</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Paid request in Department X, approved by the Teacher, parent verified (1 form).</t>
+          <t>Two requests approved by the Teacher (1 paid, 1 excused), parent verified.</t>
         </is>
       </c>
     </row>
@@ -4329,12 +4285,12 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Student 2</t>
+          <t>Student 4</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Two requests approved by the Teacher (1 paid, 1 excused), parent verified.</t>
+          <t>A request approved by the Teacher in Department Y.</t>
         </is>
       </c>
     </row>
@@ -4346,12 +4302,12 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Student 4</t>
+          <t>Student 7</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>A request approved by the Teacher in Department Y.</t>
+          <t>Excused request with a medical certificate, approved by the Teacher.</t>
         </is>
       </c>
     </row>
@@ -4363,12 +4319,12 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Student 7</t>
+          <t>Students 9 and 10</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Excused request with a medical certificate, approved by the Teacher.</t>
+          <t>Paid requests accepted, assessed and with a receipt uploaded, in Department X.</t>
         </is>
       </c>
     </row>
@@ -4380,12 +4336,12 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>Students 9 and 10</t>
+          <t>Mailboxes</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Paid requests accepted, assessed and with a receipt uploaded, in Department X.</t>
+          <t>Real inboxes for the students, Registrar and Program Head to check the emails.</t>
         </is>
       </c>
     </row>
@@ -4397,29 +4353,29 @@
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>Mailboxes</t>
+          <t>Note</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Real inboxes for the students, Registrar and Program Head to check the emails.</t>
+          <t>Many tests change data (accept, reject, return, delete, save terms). Use a test system and create fresh requests before repeating a test. Test cases name people as examples; use any account that matches the description.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Program Head</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>Note</t>
+          <t>TEST SYSTEM ONLY</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>Many tests change data (accept, reject, return, delete, save terms). Use a test system and create fresh requests before repeating a test. Test cases name people as examples; use any account that matches the description.</t>
+          <t>Several test cases delete data (Delete user, Delete department, Reset Test Data, Import School Data). Run them on a test copy of EXAMFLOW, never on the live school data.</t>
         </is>
       </c>
     </row>
@@ -4431,12 +4387,12 @@
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>TEST SYSTEM ONLY</t>
+          <t>Admin A</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Several test cases delete data (Delete user, Delete department, Reset Test Data, Import School Data). Run them on a test copy of EXAMFLOW, never on the live school data.</t>
+          <t>An active Admin account. A second Admin account (Admin B) is needed for the 'another admin' tests.</t>
         </is>
       </c>
     </row>
@@ -4448,12 +4404,12 @@
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>Admin A</t>
+          <t>Other roles</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>An active Admin account. A second Admin account (Admin B) is needed for the 'another admin' tests.</t>
+          <t>One active account for each of: Registrar, Program Head, Subject Teacher, Student (to log in as them and to check results).</t>
         </is>
       </c>
     </row>
@@ -4465,12 +4421,12 @@
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>Other roles</t>
+          <t>Requests</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>One active account for each of: Registrar, Program Head, Subject Teacher, Student (to log in as them and to check results).</t>
+          <t>Requests at every step: waiting for Teacher, Program Head first approval, assessment, payment, receipt to verify, rejected and scheduled, in at least two departments.</t>
         </is>
       </c>
     </row>
@@ -4482,12 +4438,12 @@
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>Requests</t>
+          <t>School Data files</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Requests at every step: waiting for Registrar, Teacher, Program Head first approval, assessment, payment, receipt to verify, rejected and scheduled, in at least two departments.</t>
+          <t>A correct .xlsx file with the five sheets (Departments, Programs, Staff, Students, Classes) and several broken files: missing sheet, missing column, duplicate email, bad year level (6), bad student number, class teacher not on the Staff sheet, a file over 10 MB, a .pdf, and a text file renamed .xlsx. Also import a file once so the Add User lists (student course/year/section, teacher classes) have classes to choose from.</t>
         </is>
       </c>
     </row>
@@ -4499,12 +4455,12 @@
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>School Data files</t>
+          <t>Email addresses</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>A correct .xlsx file with the five sheets (Departments, Programs, Staff, Students, Classes) and several broken files: missing sheet, missing column, duplicate email, bad year level (6), bad student number, class teacher not on the Staff sheet, a file over 10 MB, a .pdf, and a text file renamed .xlsx. Also import a file once so the Add User lists (student course/year/section, teacher classes) have classes to choose from.</t>
+          <t>Unused email addresses ending in the school domain (stamaria.sti.edu.ph) for creating test users. Accounts made with '+ Add User' have NO password: to log in as them, use a real Microsoft school account with that email.</t>
         </is>
       </c>
     </row>
@@ -4516,12 +4472,12 @@
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>Email addresses</t>
+          <t>Mailboxes</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Unused email addresses ending in the school domain (stamaria.sti.edu.ph) for creating test users. Accounts made with '+ Add User' have NO password: to log in as them, use a real Microsoft school account with that email.</t>
+          <t>Not needed for the Admin tests, except where a case says a student or Registrar is notified.</t>
         </is>
       </c>
     </row>
@@ -4533,34 +4489,17 @@
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>Mailboxes</t>
+          <t>Note</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Not needed for the Admin tests, except where a case says a student or Registrar is notified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="6" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="B51" s="6" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="C51" s="6" t="inlineStr">
-        <is>
           <t>Test cases refer to people and values as examples. Use any account that matches the description.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C51"/>
+  <autoFilter ref="A1:C50"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>